<commit_message>
excel format phne_no column
</commit_message>
<xml_diff>
--- a/storage/app/public/templates/berkumpulan.xlsx
+++ b/storage/app/public/templates/berkumpulan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/radhifauzan/Desktop/side-projects/bowling-system-backend/storage/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/radhifauzan/Desktop/side-projects/bowling-system-backend/storage/app/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F84C82CE-B80B-674D-A723-B5805627DAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{430CF5E2-BCA3-F645-85C6-55EC6E080490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -464,6 +464,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.1640625" style="1"/>
+    <col min="3" max="3" width="8.83203125" style="1"/>
     <col min="11" max="11" width="28" style="1" customWidth="1"/>
     <col min="12" max="12" width="23" customWidth="1"/>
     <col min="13" max="13" width="9.1640625" style="1"/>
@@ -540,7 +541,7 @@
       <c r="B2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D2" t="s">

</xml_diff>